<commit_message>
Actualizar checklist con las entregas de los puntos 1, 2, 4.3, 6, 9 y 14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NuMj3fWq11HABbrtni6hs7
</commit_message>
<xml_diff>
--- a/Adaptacion Plan de Estudios 2026/Checklist de entregas - Rediseño Curricular 2026.xlsx
+++ b/Adaptacion Plan de Estudios 2026/Checklist de entregas - Rediseño Curricular 2026.xlsx
@@ -731,17 +731,27 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J6" s="6" t="n">
         <v>1</v>
       </c>
@@ -769,17 +779,27 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I7" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J7" s="6" t="n">
         <v>1</v>
       </c>
@@ -807,17 +827,27 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I8" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J8" s="6" t="n">
         <v>1</v>
       </c>
@@ -845,17 +875,27 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J9" s="6" t="n">
         <v>1</v>
       </c>
@@ -883,17 +923,27 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J10" s="6" t="n">
         <v>1</v>
       </c>
@@ -921,17 +971,27 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I11" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J11" s="6" t="n">
         <v>1</v>
       </c>
@@ -959,17 +1019,27 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I12" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J12" s="6" t="n">
         <v>1</v>
       </c>
@@ -997,17 +1067,27 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J13" s="6" t="n">
         <v>1</v>
       </c>
@@ -1035,17 +1115,27 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J14" s="6" t="n">
         <v>1</v>
       </c>
@@ -1073,17 +1163,27 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I15" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J15" s="6" t="n">
         <v>1</v>
       </c>
@@ -1111,17 +1211,27 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I16" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J16" s="6" t="n">
         <v>1</v>
       </c>
@@ -1149,17 +1259,27 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I17" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1269,17 +1389,27 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J20" s="6" t="n">
         <v>1</v>
       </c>
@@ -1325,7 +1455,7 @@
       </c>
       <c r="I21" s="10" t="inlineStr">
         <is>
-          <t>Documento Misión, Visión y Perfil Profesional 2026</t>
+          <t xml:space="preserve">Documento Misión, Visión y Perfil Profesional 2026; también en Documento Primera Parte Entrega (elegir versión)</t>
         </is>
       </c>
       <c r="J21" s="6" t="n">
@@ -1411,7 +1541,7 @@
       </c>
       <c r="I23" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documento Misión, Visión y Perfil Profesional 2026; también en Documento 04 Plan de Estudios 2026</t>
+          <t xml:space="preserve">Documento Misión, Visión y Perfil Profesional 2026; también en Documento 04 Plan de Estudios 2026; también en Documento Primera Parte Entrega (elegir versión)</t>
         </is>
       </c>
       <c r="J23" s="6" t="n">
@@ -1479,17 +1609,27 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J25" s="6" t="n">
         <v>1</v>
       </c>
@@ -1517,17 +1657,27 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="n"/>
-      <c r="G26" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento Primera Parte Entrega</t>
+        </is>
+      </c>
       <c r="J26" s="6" t="n">
         <v>1</v>
       </c>
@@ -2539,17 +2689,27 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n"/>
-      <c r="G49" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I49" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I49" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plan de Estudios Propuesto para comisión v.2</t>
+        </is>
+      </c>
       <c r="J49" s="6" t="n">
         <v>1</v>
       </c>
@@ -2577,17 +2737,27 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n"/>
-      <c r="G50" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I50" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I50" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plan de Estudios Propuesto para comisión v.2</t>
+        </is>
+      </c>
       <c r="J50" s="6" t="n">
         <v>1</v>
       </c>
@@ -2633,7 +2803,7 @@
       </c>
       <c r="I51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documento 04 Plan de Estudios 2026</t>
+          <t xml:space="preserve">Documento 04 Plan de Estudios 2026; también en Plan de Estudios Propuesto para comisión v.2 (elegir versión)</t>
         </is>
       </c>
       <c r="J51" s="6" t="n">
@@ -2681,7 +2851,7 @@
       </c>
       <c r="I52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documento 04 Plan de Estudios 2026</t>
+          <t xml:space="preserve">Documento 04 Plan de Estudios 2026; también en Plan de Estudios Propuesto para comisión v.2 (elegir versión)</t>
         </is>
       </c>
       <c r="J52" s="6" t="n">
@@ -2711,17 +2881,27 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n"/>
-      <c r="G53" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I53" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I53" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plan de Estudios Propuesto para comisión v.2</t>
+        </is>
+      </c>
       <c r="J53" s="6" t="n">
         <v>1</v>
       </c>
@@ -3775,17 +3955,27 @@
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F78" s="9" t="n"/>
-      <c r="G78" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I78" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I78" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 6 Investigación</t>
+        </is>
+      </c>
       <c r="J78" s="6" t="n">
         <v>1</v>
       </c>
@@ -3813,17 +4003,27 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F79" s="9" t="n"/>
-      <c r="G79" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Word</t>
+        </is>
+      </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I79" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I79" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe Subcomisión 6 Investigación</t>
+        </is>
+      </c>
       <c r="J79" s="6" t="n">
         <v>1</v>
       </c>
@@ -4287,17 +4487,27 @@
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F91" s="9" t="n"/>
-      <c r="G91" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F91" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Excel</t>
+        </is>
+      </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I91" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I91" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Listados de bibliografía por asignatura (43) y de trabajos de grado (7), 52 archivos Excel</t>
+        </is>
+      </c>
       <c r="J91" s="6" t="n">
         <v>1</v>
       </c>
@@ -5401,17 +5611,27 @@
       </c>
       <c r="E119" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F119" s="9" t="n"/>
-      <c r="G119" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F119" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G119" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF</t>
+        </is>
+      </c>
       <c r="H119" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I119" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I119" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diagnóstico Rediseño Curricular Infraestructura (PDF)</t>
+        </is>
+      </c>
       <c r="J119" s="6" t="n">
         <v>1</v>
       </c>
@@ -5515,17 +5735,27 @@
       </c>
       <c r="E122" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F122" s="9" t="n"/>
-      <c r="G122" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F122" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G122" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF</t>
+        </is>
+      </c>
       <c r="H122" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I122" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I122" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diagnóstico Rediseño Curricular Infraestructura (PDF)</t>
+        </is>
+      </c>
       <c r="J122" s="6" t="n">
         <v>1</v>
       </c>
@@ -5553,17 +5783,27 @@
       </c>
       <c r="E123" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F123" s="9" t="n"/>
-      <c r="G123" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F123" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G123" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF</t>
+        </is>
+      </c>
       <c r="H123" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I123" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I123" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diagnóstico Rediseño Curricular Infraestructura (PDF)</t>
+        </is>
+      </c>
       <c r="J123" s="6" t="n">
         <v>1</v>
       </c>
@@ -5591,17 +5831,27 @@
       </c>
       <c r="E124" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F124" s="9" t="n"/>
-      <c r="G124" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F124" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G124" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF</t>
+        </is>
+      </c>
       <c r="H124" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I124" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I124" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diagnóstico Rediseño Curricular Infraestructura (PDF)</t>
+        </is>
+      </c>
       <c r="J124" s="6" t="n">
         <v>1</v>
       </c>
@@ -5705,17 +5955,27 @@
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F127" s="9" t="n"/>
-      <c r="G127" s="6" t="n"/>
+          <t xml:space="preserve">Entregado</t>
+        </is>
+      </c>
+      <c r="F127" s="9" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G127" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF</t>
+        </is>
+      </c>
       <c r="H127" s="6" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I127" s="10" t="n"/>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="I127" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diagnóstico Rediseño Curricular Infraestructura (PDF)</t>
+        </is>
+      </c>
       <c r="J127" s="6" t="n">
         <v>1</v>
       </c>

</xml_diff>